<commit_message>
Start content calendar and KPI weeks on 19 November 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012aVsoCbqH8naSiNgykD1Dt
</commit_message>
<xml_diff>
--- a/yontro-sheets/Yontro Content & Uploads.xlsx
+++ b/yontro-sheets/Yontro Content & Uploads.xlsx
@@ -116,7 +116,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">T-YYYYMMDD-PAGE-n, e.g. T-20261027-FT-1</t>
+          <t xml:space="preserve">T-YYYYMMDD-PAGE-n, e.g. T-20261119-FT-1</t>
         </r>
       </text>
     </comment>
@@ -479,7 +479,7 @@
     <t xml:space="preserve">Hook line</t>
   </si>
   <si>
-    <t xml:space="preserve">FT_20261026_1_A</t>
+    <t xml:space="preserve">FT_20261118_1_A</t>
   </si>
   <si>
     <t xml:space="preserve">Posted</t>
@@ -548,7 +548,7 @@
     <t xml:space="preserve">EXAMPLE: He lost everything at 48</t>
   </si>
   <si>
-    <t xml:space="preserve">T-20261024-FT-1</t>
+    <t xml:space="preserve">T-20261117-FT-1</t>
   </si>
   <si>
     <t xml:space="preserve">Azeem</t>
@@ -656,7 +656,7 @@
     <t xml:space="preserve">Active</t>
   </si>
   <si>
-    <t xml:space="preserve">Week start (Mon)</t>
+    <t xml:space="preserve">Week start</t>
   </si>
   <si>
     <t xml:space="preserve">Week end</t>
@@ -1600,7 +1600,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="n">
-        <v>46321</v>
+        <v>46344</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>31</v>
@@ -1633,7 +1633,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>38</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>38</v>
@@ -1683,7 +1683,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>38</v>
@@ -1708,7 +1708,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>41</v>
@@ -1733,7 +1733,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>41</v>
@@ -1758,7 +1758,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>41</v>
@@ -1783,7 +1783,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>31</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>31</v>
@@ -1833,7 +1833,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
-        <v>46322</v>
+        <v>46345</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>31</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>38</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>38</v>
@@ -1908,7 +1908,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>38</v>
@@ -1933,7 +1933,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>41</v>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>41</v>
@@ -1983,7 +1983,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>41</v>
@@ -2008,7 +2008,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>31</v>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>31</v>
@@ -2058,7 +2058,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="n">
-        <v>46323</v>
+        <v>46346</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>31</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>38</v>
@@ -2108,7 +2108,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>38</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>38</v>
@@ -2158,7 +2158,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>41</v>
@@ -2183,7 +2183,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>41</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>41</v>
@@ -2233,7 +2233,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>31</v>
@@ -2258,7 +2258,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>31</v>
@@ -2283,7 +2283,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="n">
-        <v>46324</v>
+        <v>46347</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>31</v>
@@ -2308,7 +2308,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>38</v>
@@ -2333,7 +2333,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>38</v>
@@ -2358,7 +2358,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>38</v>
@@ -2383,7 +2383,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>41</v>
@@ -2408,7 +2408,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>41</v>
@@ -2433,7 +2433,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>41</v>
@@ -2458,7 +2458,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>31</v>
@@ -2483,7 +2483,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>31</v>
@@ -2508,7 +2508,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="n">
-        <v>46325</v>
+        <v>46348</v>
       </c>
       <c r="B38" s="12" t="s">
         <v>31</v>
@@ -2533,7 +2533,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B39" s="12" t="s">
         <v>38</v>
@@ -2558,7 +2558,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B40" s="12" t="s">
         <v>38</v>
@@ -2583,7 +2583,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>38</v>
@@ -2608,7 +2608,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B42" s="12" t="s">
         <v>41</v>
@@ -2633,7 +2633,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B43" s="12" t="s">
         <v>41</v>
@@ -2658,7 +2658,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B44" s="12" t="s">
         <v>41</v>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B45" s="12" t="s">
         <v>31</v>
@@ -2708,7 +2708,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B46" s="12" t="s">
         <v>31</v>
@@ -2733,7 +2733,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="n">
-        <v>46326</v>
+        <v>46349</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>31</v>
@@ -2758,7 +2758,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>38</v>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>38</v>
@@ -2808,7 +2808,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B50" s="12" t="s">
         <v>38</v>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B51" s="12" t="s">
         <v>41</v>
@@ -2858,7 +2858,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B52" s="12" t="s">
         <v>41</v>
@@ -2883,7 +2883,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B53" s="12" t="s">
         <v>41</v>
@@ -2908,7 +2908,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B54" s="12" t="s">
         <v>31</v>
@@ -2933,7 +2933,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>31</v>
@@ -2958,7 +2958,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="n">
-        <v>46327</v>
+        <v>46350</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>31</v>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B57" s="12" t="s">
         <v>38</v>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B58" s="12" t="s">
         <v>38</v>
@@ -3033,7 +3033,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B59" s="12" t="s">
         <v>38</v>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B60" s="12" t="s">
         <v>41</v>
@@ -3083,7 +3083,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B61" s="12" t="s">
         <v>41</v>
@@ -3108,7 +3108,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B62" s="12" t="s">
         <v>41</v>
@@ -3133,7 +3133,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B63" s="12" t="s">
         <v>31</v>
@@ -3158,7 +3158,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B64" s="12" t="s">
         <v>31</v>
@@ -3183,7 +3183,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="n">
-        <v>46328</v>
+        <v>46351</v>
       </c>
       <c r="B65" s="12" t="s">
         <v>31</v>
@@ -3208,7 +3208,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B66" s="12" t="s">
         <v>38</v>
@@ -3233,7 +3233,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B67" s="12" t="s">
         <v>38</v>
@@ -3258,7 +3258,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B68" s="12" t="s">
         <v>38</v>
@@ -3283,7 +3283,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B69" s="12" t="s">
         <v>41</v>
@@ -3308,7 +3308,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B70" s="12" t="s">
         <v>41</v>
@@ -3333,7 +3333,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B71" s="12" t="s">
         <v>41</v>
@@ -3358,7 +3358,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B72" s="12" t="s">
         <v>31</v>
@@ -3383,7 +3383,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B73" s="12" t="s">
         <v>31</v>
@@ -3408,7 +3408,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="11" t="n">
-        <v>46329</v>
+        <v>46352</v>
       </c>
       <c r="B74" s="12" t="s">
         <v>31</v>
@@ -3433,7 +3433,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B75" s="12" t="s">
         <v>38</v>
@@ -3458,7 +3458,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B76" s="12" t="s">
         <v>38</v>
@@ -3483,7 +3483,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B77" s="12" t="s">
         <v>38</v>
@@ -3508,7 +3508,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B78" s="12" t="s">
         <v>41</v>
@@ -3533,7 +3533,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B79" s="12" t="s">
         <v>41</v>
@@ -3558,7 +3558,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B80" s="12" t="s">
         <v>41</v>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B81" s="12" t="s">
         <v>31</v>
@@ -3608,7 +3608,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>31</v>
@@ -3633,7 +3633,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="n">
-        <v>46330</v>
+        <v>46353</v>
       </c>
       <c r="B83" s="12" t="s">
         <v>31</v>
@@ -3658,7 +3658,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B84" s="12" t="s">
         <v>38</v>
@@ -3683,7 +3683,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B85" s="12" t="s">
         <v>38</v>
@@ -3708,7 +3708,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B86" s="12" t="s">
         <v>38</v>
@@ -3733,7 +3733,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B87" s="12" t="s">
         <v>41</v>
@@ -3758,7 +3758,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>41</v>
@@ -3783,7 +3783,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B89" s="12" t="s">
         <v>41</v>
@@ -3808,7 +3808,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B90" s="12" t="s">
         <v>31</v>
@@ -3833,7 +3833,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B91" s="12" t="s">
         <v>31</v>
@@ -3858,7 +3858,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="n">
-        <v>46331</v>
+        <v>46354</v>
       </c>
       <c r="B92" s="12" t="s">
         <v>31</v>
@@ -3883,7 +3883,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B93" s="12" t="s">
         <v>38</v>
@@ -3908,7 +3908,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B94" s="12" t="s">
         <v>38</v>
@@ -3933,7 +3933,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B95" s="12" t="s">
         <v>38</v>
@@ -3958,7 +3958,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>41</v>
@@ -3983,7 +3983,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B97" s="12" t="s">
         <v>41</v>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B98" s="12" t="s">
         <v>41</v>
@@ -4033,7 +4033,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B99" s="12" t="s">
         <v>31</v>
@@ -4058,7 +4058,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B100" s="12" t="s">
         <v>31</v>
@@ -4083,7 +4083,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="n">
-        <v>46332</v>
+        <v>46355</v>
       </c>
       <c r="B101" s="12" t="s">
         <v>31</v>
@@ -4108,7 +4108,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B102" s="12" t="s">
         <v>38</v>
@@ -4133,7 +4133,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B103" s="12" t="s">
         <v>38</v>
@@ -4158,7 +4158,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B104" s="12" t="s">
         <v>38</v>
@@ -4183,7 +4183,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B105" s="12" t="s">
         <v>41</v>
@@ -4208,7 +4208,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B106" s="12" t="s">
         <v>41</v>
@@ -4233,7 +4233,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B107" s="12" t="s">
         <v>41</v>
@@ -4258,7 +4258,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B108" s="12" t="s">
         <v>31</v>
@@ -4283,7 +4283,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B109" s="12" t="s">
         <v>31</v>
@@ -4308,7 +4308,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="11" t="n">
-        <v>46333</v>
+        <v>46356</v>
       </c>
       <c r="B110" s="12" t="s">
         <v>31</v>
@@ -4333,7 +4333,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B111" s="12" t="s">
         <v>38</v>
@@ -4358,7 +4358,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B112" s="12" t="s">
         <v>38</v>
@@ -4383,7 +4383,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>38</v>
@@ -4408,7 +4408,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B114" s="12" t="s">
         <v>41</v>
@@ -4433,7 +4433,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B115" s="12" t="s">
         <v>41</v>
@@ -4458,7 +4458,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B116" s="12" t="s">
         <v>41</v>
@@ -4483,7 +4483,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B117" s="12" t="s">
         <v>31</v>
@@ -4508,7 +4508,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B118" s="12" t="s">
         <v>31</v>
@@ -4533,7 +4533,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="n">
-        <v>46334</v>
+        <v>46357</v>
       </c>
       <c r="B119" s="12" t="s">
         <v>31</v>
@@ -4558,7 +4558,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B120" s="12" t="s">
         <v>38</v>
@@ -4583,7 +4583,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B121" s="12" t="s">
         <v>38</v>
@@ -4608,7 +4608,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B122" s="12" t="s">
         <v>38</v>
@@ -4633,7 +4633,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B123" s="12" t="s">
         <v>41</v>
@@ -4658,7 +4658,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B124" s="12" t="s">
         <v>41</v>
@@ -4683,7 +4683,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B125" s="12" t="s">
         <v>41</v>
@@ -4708,7 +4708,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B126" s="12" t="s">
         <v>31</v>
@@ -4733,7 +4733,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B127" s="12" t="s">
         <v>31</v>
@@ -4758,7 +4758,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="11" t="n">
-        <v>46335</v>
+        <v>46358</v>
       </c>
       <c r="B128" s="12" t="s">
         <v>31</v>
@@ -4908,7 +4908,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="n">
-        <v>46320</v>
+        <v>46344</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>31</v>
@@ -15067,7 +15067,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="8" t="n">
-        <v>46319</v>
+        <v>46343</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>31</v>
@@ -15125,7 +15125,7 @@
         <v>Yes: add to Constants</v>
       </c>
       <c r="T2" s="8" t="n">
-        <v>46320</v>
+        <v>46344</v>
       </c>
       <c r="U2" s="9"/>
     </row>
@@ -29177,7 +29177,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="n">
-        <v>46320</v>
+        <v>46344</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>35</v>
@@ -31675,11 +31675,11 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="n">
-        <v>46321</v>
+        <v>46345</v>
       </c>
       <c r="B2" s="22" t="n">
         <f aca="false">IF(A2="","",A2+6)</f>
-        <v>46327</v>
+        <v>46351</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>38</v>
@@ -31731,11 +31731,11 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="n">
-        <v>46321</v>
+        <v>46345</v>
       </c>
       <c r="B3" s="22" t="n">
         <f aca="false">IF(A3="","",A3+6)</f>
-        <v>46327</v>
+        <v>46351</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>41</v>
@@ -31787,11 +31787,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="n">
-        <v>46321</v>
+        <v>46345</v>
       </c>
       <c r="B4" s="22" t="n">
         <f aca="false">IF(A4="","",A4+6)</f>
-        <v>46327</v>
+        <v>46351</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>31</v>
@@ -31843,11 +31843,11 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="n">
-        <v>46328</v>
+        <v>46352</v>
       </c>
       <c r="B5" s="22" t="n">
         <f aca="false">IF(A5="","",A5+6)</f>
-        <v>46334</v>
+        <v>46358</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>38</v>
@@ -31899,11 +31899,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
-        <v>46328</v>
+        <v>46352</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">IF(A6="","",A6+6)</f>
-        <v>46334</v>
+        <v>46358</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>41</v>
@@ -31955,11 +31955,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
-        <v>46328</v>
+        <v>46352</v>
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">IF(A7="","",A7+6)</f>
-        <v>46334</v>
+        <v>46358</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>31</v>
@@ -32011,11 +32011,11 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
-        <v>46335</v>
+        <v>46359</v>
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">IF(A8="","",A8+6)</f>
-        <v>46341</v>
+        <v>46365</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>38</v>
@@ -32067,11 +32067,11 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
-        <v>46335</v>
+        <v>46359</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">IF(A9="","",A9+6)</f>
-        <v>46341</v>
+        <v>46365</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>41</v>
@@ -32123,11 +32123,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
-        <v>46335</v>
+        <v>46359</v>
       </c>
       <c r="B10" s="22" t="n">
         <f aca="false">IF(A10="","",A10+6)</f>
-        <v>46341</v>
+        <v>46365</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>31</v>
@@ -32179,11 +32179,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
-        <v>46342</v>
+        <v>46366</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">IF(A11="","",A11+6)</f>
-        <v>46348</v>
+        <v>46372</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>38</v>
@@ -32235,11 +32235,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="n">
-        <v>46342</v>
+        <v>46366</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">IF(A12="","",A12+6)</f>
-        <v>46348</v>
+        <v>46372</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>41</v>
@@ -32291,11 +32291,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
-        <v>46342</v>
+        <v>46366</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">IF(A13="","",A13+6)</f>
-        <v>46348</v>
+        <v>46372</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>31</v>
@@ -32347,11 +32347,11 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="n">
-        <v>46349</v>
+        <v>46373</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">IF(A14="","",A14+6)</f>
-        <v>46355</v>
+        <v>46379</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>38</v>
@@ -32403,11 +32403,11 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
-        <v>46349</v>
+        <v>46373</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">IF(A15="","",A15+6)</f>
-        <v>46355</v>
+        <v>46379</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>41</v>
@@ -32459,11 +32459,11 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
-        <v>46349</v>
+        <v>46373</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">IF(A16="","",A16+6)</f>
-        <v>46355</v>
+        <v>46379</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>31</v>
@@ -32515,11 +32515,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
-        <v>46356</v>
+        <v>46380</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">IF(A17="","",A17+6)</f>
-        <v>46362</v>
+        <v>46386</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>38</v>
@@ -32571,11 +32571,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="n">
-        <v>46356</v>
+        <v>46380</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">IF(A18="","",A18+6)</f>
-        <v>46362</v>
+        <v>46386</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>41</v>
@@ -32627,11 +32627,11 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="n">
-        <v>46356</v>
+        <v>46380</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">IF(A19="","",A19+6)</f>
-        <v>46362</v>
+        <v>46386</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>31</v>
@@ -32683,11 +32683,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="n">
-        <v>46363</v>
+        <v>46387</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">IF(A20="","",A20+6)</f>
-        <v>46369</v>
+        <v>46393</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>38</v>
@@ -32739,11 +32739,11 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="n">
-        <v>46363</v>
+        <v>46387</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">IF(A21="","",A21+6)</f>
-        <v>46369</v>
+        <v>46393</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>41</v>
@@ -32795,11 +32795,11 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="n">
-        <v>46363</v>
+        <v>46387</v>
       </c>
       <c r="B22" s="22" t="n">
         <f aca="false">IF(A22="","",A22+6)</f>
-        <v>46369</v>
+        <v>46393</v>
       </c>
       <c r="C22" s="12" t="s">
         <v>31</v>
@@ -32851,11 +32851,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="n">
-        <v>46370</v>
+        <v>46394</v>
       </c>
       <c r="B23" s="22" t="n">
         <f aca="false">IF(A23="","",A23+6)</f>
-        <v>46376</v>
+        <v>46400</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>38</v>
@@ -32907,11 +32907,11 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="n">
-        <v>46370</v>
+        <v>46394</v>
       </c>
       <c r="B24" s="22" t="n">
         <f aca="false">IF(A24="","",A24+6)</f>
-        <v>46376</v>
+        <v>46400</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>41</v>
@@ -32963,11 +32963,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="n">
-        <v>46370</v>
+        <v>46394</v>
       </c>
       <c r="B25" s="22" t="n">
         <f aca="false">IF(A25="","",A25+6)</f>
-        <v>46376</v>
+        <v>46400</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>31</v>
@@ -33019,11 +33019,11 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="n">
-        <v>46377</v>
+        <v>46401</v>
       </c>
       <c r="B26" s="22" t="n">
         <f aca="false">IF(A26="","",A26+6)</f>
-        <v>46383</v>
+        <v>46407</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>38</v>
@@ -33075,11 +33075,11 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="n">
-        <v>46377</v>
+        <v>46401</v>
       </c>
       <c r="B27" s="22" t="n">
         <f aca="false">IF(A27="","",A27+6)</f>
-        <v>46383</v>
+        <v>46407</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>41</v>
@@ -33131,11 +33131,11 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
-        <v>46377</v>
+        <v>46401</v>
       </c>
       <c r="B28" s="22" t="n">
         <f aca="false">IF(A28="","",A28+6)</f>
-        <v>46383</v>
+        <v>46407</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>31</v>
@@ -33187,11 +33187,11 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="n">
-        <v>46384</v>
+        <v>46408</v>
       </c>
       <c r="B29" s="22" t="n">
         <f aca="false">IF(A29="","",A29+6)</f>
-        <v>46390</v>
+        <v>46414</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>38</v>
@@ -33243,11 +33243,11 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
-        <v>46384</v>
+        <v>46408</v>
       </c>
       <c r="B30" s="22" t="n">
         <f aca="false">IF(A30="","",A30+6)</f>
-        <v>46390</v>
+        <v>46414</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>41</v>
@@ -33299,11 +33299,11 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="n">
-        <v>46384</v>
+        <v>46408</v>
       </c>
       <c r="B31" s="22" t="n">
         <f aca="false">IF(A31="","",A31+6)</f>
-        <v>46390</v>
+        <v>46414</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>31</v>
@@ -33355,11 +33355,11 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="n">
-        <v>46391</v>
+        <v>46415</v>
       </c>
       <c r="B32" s="22" t="n">
         <f aca="false">IF(A32="","",A32+6)</f>
-        <v>46397</v>
+        <v>46421</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>38</v>
@@ -33411,11 +33411,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="n">
-        <v>46391</v>
+        <v>46415</v>
       </c>
       <c r="B33" s="22" t="n">
         <f aca="false">IF(A33="","",A33+6)</f>
-        <v>46397</v>
+        <v>46421</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>41</v>
@@ -33467,11 +33467,11 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="n">
-        <v>46391</v>
+        <v>46415</v>
       </c>
       <c r="B34" s="22" t="n">
         <f aca="false">IF(A34="","",A34+6)</f>
-        <v>46397</v>
+        <v>46421</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>31</v>
@@ -33523,11 +33523,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="n">
-        <v>46398</v>
+        <v>46422</v>
       </c>
       <c r="B35" s="22" t="n">
         <f aca="false">IF(A35="","",A35+6)</f>
-        <v>46404</v>
+        <v>46428</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>38</v>
@@ -33579,11 +33579,11 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="n">
-        <v>46398</v>
+        <v>46422</v>
       </c>
       <c r="B36" s="22" t="n">
         <f aca="false">IF(A36="","",A36+6)</f>
-        <v>46404</v>
+        <v>46428</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>41</v>
@@ -33635,11 +33635,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="n">
-        <v>46398</v>
+        <v>46422</v>
       </c>
       <c r="B37" s="22" t="n">
         <f aca="false">IF(A37="","",A37+6)</f>
-        <v>46404</v>
+        <v>46428</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>31</v>
@@ -35016,11 +35016,11 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="n">
-        <v>46321</v>
+        <v>46345</v>
       </c>
       <c r="B2" s="22" t="n">
         <f aca="false">IF(A2="","",A2+6)</f>
-        <v>46327</v>
+        <v>46351</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="19" t="str">
@@ -35055,11 +35055,11 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="n">
-        <v>46328</v>
+        <v>46352</v>
       </c>
       <c r="B3" s="22" t="n">
         <f aca="false">IF(A3="","",A3+6)</f>
-        <v>46334</v>
+        <v>46358</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="19" t="str">
@@ -35094,11 +35094,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="n">
-        <v>46335</v>
+        <v>46359</v>
       </c>
       <c r="B4" s="22" t="n">
         <f aca="false">IF(A4="","",A4+6)</f>
-        <v>46341</v>
+        <v>46365</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="19" t="str">
@@ -35133,11 +35133,11 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="n">
-        <v>46342</v>
+        <v>46366</v>
       </c>
       <c r="B5" s="22" t="n">
         <f aca="false">IF(A5="","",A5+6)</f>
-        <v>46348</v>
+        <v>46372</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="19" t="str">
@@ -35172,11 +35172,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
-        <v>46349</v>
+        <v>46373</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">IF(A6="","",A6+6)</f>
-        <v>46355</v>
+        <v>46379</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="19" t="str">
@@ -35211,11 +35211,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
-        <v>46356</v>
+        <v>46380</v>
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">IF(A7="","",A7+6)</f>
-        <v>46362</v>
+        <v>46386</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="19" t="str">
@@ -35250,11 +35250,11 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
-        <v>46363</v>
+        <v>46387</v>
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">IF(A8="","",A8+6)</f>
-        <v>46369</v>
+        <v>46393</v>
       </c>
       <c r="C8" s="17"/>
       <c r="D8" s="19" t="str">
@@ -35289,11 +35289,11 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
-        <v>46370</v>
+        <v>46394</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">IF(A9="","",A9+6)</f>
-        <v>46376</v>
+        <v>46400</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="19" t="str">
@@ -35328,11 +35328,11 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
-        <v>46377</v>
+        <v>46401</v>
       </c>
       <c r="B10" s="22" t="n">
         <f aca="false">IF(A10="","",A10+6)</f>
-        <v>46383</v>
+        <v>46407</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="19" t="str">
@@ -35367,11 +35367,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
-        <v>46384</v>
+        <v>46408</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">IF(A11="","",A11+6)</f>
-        <v>46390</v>
+        <v>46414</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="19" t="str">
@@ -35406,11 +35406,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="n">
-        <v>46391</v>
+        <v>46415</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">IF(A12="","",A12+6)</f>
-        <v>46397</v>
+        <v>46421</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="19" t="str">
@@ -35445,11 +35445,11 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
-        <v>46398</v>
+        <v>46422</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">IF(A13="","",A13+6)</f>
-        <v>46404</v>
+        <v>46428</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="19" t="str">

</xml_diff>